<commit_message>
"update docs + readme "
</commit_message>
<xml_diff>
--- a/docs/Manual_Test_Cases.xlsx
+++ b/docs/Manual_Test_Cases.xlsx
@@ -1430,7 +1430,7 @@
 
 <file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1447,85 +1447,54 @@
     <col min="12" max="12" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
+    <row r="1" spans="1:12">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>E2E Playwright Automation Framework - Danh sach test case manual</t>
+        </is>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="I2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="J2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="K2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="L2" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -1534,22 +1503,22 @@
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="H3" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="I3" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="J3" t="s">
         <v>21</v>
@@ -1558,36 +1527,36 @@
         <v>22</v>
       </c>
       <c r="L3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
         <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="I4" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="J4" t="s">
         <v>21</v>
@@ -1596,12 +1565,12 @@
         <v>22</v>
       </c>
       <c r="L4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
@@ -1613,19 +1582,19 @@
         <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
         <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
         <v>36</v>
       </c>
       <c r="I5" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="J5" t="s">
         <v>21</v>
@@ -1639,31 +1608,31 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F6" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I6" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J6" t="s">
         <v>21</v>
@@ -1672,12 +1641,12 @@
         <v>22</v>
       </c>
       <c r="L6" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
@@ -1689,19 +1658,19 @@
         <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="F7" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="G7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="I7" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="J7" t="s">
         <v>21</v>
@@ -1715,31 +1684,31 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F8" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G8" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I8" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="J8" t="s">
         <v>21</v>
@@ -1753,7 +1722,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
@@ -1765,25 +1734,25 @@
         <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
         <v>59</v>
       </c>
       <c r="G9" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H9" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="I9" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="J9" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="K9" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="L9" t="s">
         <v>30</v>
@@ -1791,45 +1760,45 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="I10" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="J10" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="K10" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="L10" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B11" t="s">
         <v>69</v>
@@ -1841,33 +1810,33 @@
         <v>15</v>
       </c>
       <c r="E11" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F11" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="H11" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I11" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="J11" t="s">
         <v>21</v>
       </c>
       <c r="K11" t="s">
-        <v>81</v>
+        <v>22</v>
       </c>
       <c r="L11" t="s">
-        <v>82</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
         <v>69</v>
@@ -1879,16 +1848,16 @@
         <v>15</v>
       </c>
       <c r="E12" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F12" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="G12" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="H12" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="I12" t="s">
         <v>80</v>
@@ -1897,15 +1866,15 @@
         <v>21</v>
       </c>
       <c r="K12" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="L12" t="s">
-        <v>30</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B13" t="s">
         <v>69</v>
@@ -1917,16 +1886,16 @@
         <v>15</v>
       </c>
       <c r="E13" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G13" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H13" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="I13" t="s">
         <v>80</v>
@@ -1943,37 +1912,37 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B14" t="s">
         <v>69</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E14" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F14" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="G14" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="H14" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="I14" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="J14" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="K14" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="L14" t="s">
         <v>30</v>
@@ -1981,7 +1950,7 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B15" t="s">
         <v>69</v>
@@ -1993,19 +1962,19 @@
         <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="F15" t="s">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="G15" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="H15" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="I15" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="J15" t="s">
         <v>38</v>
@@ -2019,45 +1988,45 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B16" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E16" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="F16" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G16" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="H16" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="I16" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="J16" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="K16" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="L16" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
         <v>105</v>
@@ -2069,19 +2038,19 @@
         <v>15</v>
       </c>
       <c r="E17" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="F17" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="G17" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="H17" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="I17" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="J17" t="s">
         <v>21</v>
@@ -2090,42 +2059,42 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B18" t="s">
         <v>105</v>
       </c>
       <c r="C18" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E18" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="F18" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="G18" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="H18" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I18" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="J18" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="K18" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="L18" t="s">
         <v>30</v>
@@ -2133,7 +2102,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B19" t="s">
         <v>105</v>
@@ -2145,19 +2114,19 @@
         <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="F19" t="s">
         <v>107</v>
       </c>
       <c r="G19" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="H19" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="I19" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="J19" t="s">
         <v>38</v>
@@ -2171,7 +2140,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B20" t="s">
         <v>105</v>
@@ -2183,19 +2152,19 @@
         <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F20" t="s">
         <v>107</v>
       </c>
       <c r="G20" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="H20" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="I20" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="J20" t="s">
         <v>38</v>
@@ -2209,7 +2178,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B21" t="s">
         <v>105</v>
@@ -2221,19 +2190,19 @@
         <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F21" t="s">
         <v>107</v>
       </c>
       <c r="G21" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H21" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I21" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="J21" t="s">
         <v>38</v>
@@ -2247,45 +2216,45 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B22" t="s">
-        <v>138</v>
+        <v>105</v>
       </c>
       <c r="C22" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D22" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E22" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F22" t="s">
-        <v>140</v>
+        <v>107</v>
       </c>
       <c r="G22" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="H22" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="I22" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="J22" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="K22" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="L22" t="s">
-        <v>144</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B23" t="s">
         <v>138</v>
@@ -2297,16 +2266,16 @@
         <v>15</v>
       </c>
       <c r="E23" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F23" t="s">
         <v>140</v>
       </c>
       <c r="G23" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="H23" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="I23" t="s">
         <v>143</v>
@@ -2323,7 +2292,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B24" t="s">
         <v>138</v>
@@ -2335,16 +2304,16 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="F24" t="s">
         <v>140</v>
       </c>
       <c r="G24" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="H24" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="I24" t="s">
         <v>143</v>
@@ -2356,33 +2325,33 @@
         <v>22</v>
       </c>
       <c r="L24" t="s">
-        <v>30</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B25" t="s">
         <v>138</v>
       </c>
       <c r="C25" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D25" t="s">
         <v>15</v>
       </c>
       <c r="E25" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="F25" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="G25" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="H25" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="I25" t="s">
         <v>143</v>
@@ -2399,37 +2368,37 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B26" t="s">
-        <v>159</v>
+        <v>138</v>
       </c>
       <c r="C26" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D26" t="s">
-        <v>160</v>
+        <v>15</v>
       </c>
       <c r="E26" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="F26" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="G26" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="H26" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="I26" t="s">
         <v>143</v>
       </c>
       <c r="J26" t="s">
-        <v>165</v>
+        <v>21</v>
       </c>
       <c r="K26" t="s">
-        <v>166</v>
+        <v>22</v>
       </c>
       <c r="L26" t="s">
         <v>30</v>
@@ -2437,28 +2406,28 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="B27" t="s">
         <v>159</v>
       </c>
       <c r="C27" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D27" t="s">
         <v>160</v>
       </c>
       <c r="E27" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="F27" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="G27" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="H27" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="I27" t="s">
         <v>143</v>
@@ -2475,7 +2444,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B28" t="s">
         <v>159</v>
@@ -2487,19 +2456,19 @@
         <v>160</v>
       </c>
       <c r="E28" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="F28" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="G28" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="H28" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="I28" t="s">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="J28" t="s">
         <v>165</v>
@@ -2513,7 +2482,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B29" t="s">
         <v>159</v>
@@ -2525,19 +2494,19 @@
         <v>160</v>
       </c>
       <c r="E29" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="F29" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="G29" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="I29" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="J29" t="s">
         <v>165</v>
@@ -2549,8 +2518,232 @@
         <v>30</v>
       </c>
     </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>178</v>
+      </c>
+      <c r="B30" t="s">
+        <v>159</v>
+      </c>
+      <c r="C30" t="s">
+        <v>32</v>
+      </c>
+      <c r="D30" t="s">
+        <v>160</v>
+      </c>
+      <c r="E30" t="s">
+        <v>179</v>
+      </c>
+      <c r="F30" t="s">
+        <v>180</v>
+      </c>
+      <c r="G30" t="s">
+        <v>181</v>
+      </c>
+      <c r="H30" t="s">
+        <v>182</v>
+      </c>
+      <c r="I30" t="s">
+        <v>183</v>
+      </c>
+      <c r="J30" t="s">
+        <v>165</v>
+      </c>
+      <c r="K30" t="s">
+        <v>166</v>
+      </c>
+      <c r="L30" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>FRAME-001</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Frames</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Kiem tra noi dung trong ca hai frame</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Nguoi dung dang o trang Frames</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>1. Mo trang Frames`n2. Doc sample heading trong frame1 va frame2</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Ca hai frame hien thi This is a sample page</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Smoke case</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>FRAME-002</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Frames</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Kiem tra kich thuoc frame lon va frame nho</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Nguoi dung dang o trang Frames</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>1. Mo trang Frames`n2. So sanh bounding box cua frame1 va frame2</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Chieu rong va chieu cao cua frame thu nhat lon hon frame thu hai</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FRAME-003</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Nested Frames</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Kiem tra noi dung trong nested frames</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Nguoi dung dang o trang Nested Frames</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>1. Mo trang Nested Frames`n2. Doc noi dung parent frame`n3. Doc noi dung child iframe</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Parent frame hien thi Parent frame va child iframe hien thi Child Iframe</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Dung nested frameLocator</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L29"/>
+  <autoFilter ref="A2:L33"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>